<commit_message>
Add MDFoods Figma guidance and update profile requirements
</commit_message>
<xml_diff>
--- a/products/product_plan.xlsx
+++ b/products/product_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longtran/codes/bplatform/platform-ecosystem-docs/products/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0CAE744-B32C-B045-96CD-E96006384C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CC664D3-29CD-C34C-81E8-158088BF47B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Project / Feature</t>
   </si>
@@ -32,6 +32,12 @@
     <t>◆ v1: User can see all products/contents</t>
   </si>
   <si>
+    <t>◆ v2: User can request a quote</t>
+  </si>
+  <si>
+    <t>◆ v3: User can complete an order</t>
+  </si>
+  <si>
     <t>F-01: Master Layout</t>
   </si>
   <si>
@@ -87,6 +93,9 @@
   </si>
   <si>
     <t>F-19: In-App Messages and Notification</t>
+  </si>
+  <si>
+    <t>F-20: Password Recovery</t>
   </si>
   <si>
     <t>CRM</t>
@@ -123,7 +132,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -159,8 +168,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -185,8 +201,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -194,12 +215,81 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -215,12 +305,52 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -550,13 +680,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:EU29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="B2:EU30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelRow="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.6640625" customWidth="1"/>
     <col min="2" max="2" width="43.1640625" customWidth="1"/>
     <col min="3" max="3" width="5.83203125" style="2" customWidth="1"/>
-    <col min="4" max="151" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="151" width="5.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:151" x14ac:dyDescent="0.2">
@@ -1018,133 +1149,222 @@
       <c r="C3" s="6" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="2:151" x14ac:dyDescent="0.2">
+      <c r="X3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE3" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B4" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="2:151" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B5" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="2:151" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B6" s="8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="2:151" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B7" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="2:151" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B8" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="2:151" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B9" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="2:151" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B10" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="2:151" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B11" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="2:151" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+      <c r="D11" s="13"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="I11" s="15"/>
+    </row>
+    <row r="12" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B12" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="2:151" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="12"/>
+    </row>
+    <row r="13" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B13" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="2:151" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+      <c r="K13" s="10"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="12"/>
+    </row>
+    <row r="14" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B14" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="2:151" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+      <c r="K14" s="10"/>
+      <c r="L14" s="12"/>
+    </row>
+    <row r="15" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B15" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="2:151" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+      <c r="M15" s="10"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="12"/>
+    </row>
+    <row r="16" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B16" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="R16" s="10"/>
+      <c r="S16" s="11"/>
+      <c r="T16" s="11"/>
+      <c r="U16" s="11"/>
+      <c r="V16" s="11"/>
+      <c r="W16" s="12"/>
+    </row>
+    <row r="17" spans="2:30" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B17" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+      <c r="K17" s="10"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="12"/>
+    </row>
+    <row r="18" spans="2:30" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B18" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+      <c r="R18" s="10"/>
+      <c r="S18" s="11"/>
+      <c r="T18" s="12"/>
+    </row>
+    <row r="19" spans="2:30" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B19" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
+        <v>20</v>
+      </c>
+      <c r="U19" s="10"/>
+      <c r="V19" s="11"/>
+      <c r="W19" s="12"/>
+    </row>
+    <row r="20" spans="2:30" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B20" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+      <c r="Y20" s="10"/>
+      <c r="Z20" s="11"/>
+      <c r="AA20" s="11"/>
+      <c r="AB20" s="11"/>
+      <c r="AC20" s="12"/>
+    </row>
+    <row r="21" spans="2:30" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="Y21" s="10"/>
+      <c r="Z21" s="12"/>
+    </row>
+    <row r="22" spans="2:30" outlineLevel="1" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B24" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C24" s="6"/>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B25" s="7"/>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B26" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C26" s="6"/>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B27" s="7"/>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B28" s="1" t="s">
+      <c r="Y22" s="10"/>
+      <c r="Z22" s="11"/>
+      <c r="AA22" s="11"/>
+      <c r="AB22" s="11"/>
+      <c r="AC22" s="11"/>
+      <c r="AD22" s="12"/>
+    </row>
+    <row r="23" spans="2:30" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="6"/>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B29" s="7"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="12"/>
+    </row>
+    <row r="25" spans="2:30" x14ac:dyDescent="0.2">
+      <c r="B25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="6"/>
+    </row>
+    <row r="26" spans="2:30" x14ac:dyDescent="0.2">
+      <c r="B26" s="7"/>
+    </row>
+    <row r="27" spans="2:30" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="6"/>
+    </row>
+    <row r="28" spans="2:30" x14ac:dyDescent="0.2">
+      <c r="B28" s="7"/>
+    </row>
+    <row r="29" spans="2:30" x14ac:dyDescent="0.2">
+      <c r="B29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="6"/>
+    </row>
+    <row r="30" spans="2:30" x14ac:dyDescent="0.2">
+      <c r="B30" s="7"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:EU14 C15:L15 Q15 V15:EU15 C16:EU18 C19:Q19 X19:EU19 C20:EU21 C22:X22 AE22 AL22:EU22 C23:EU1048576">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>WEEKDAY(C$2)=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M15:P15">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>WEEKDAY(R$2)=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U19:W19">
+    <cfRule type="expression" dxfId="1" priority="5">
+      <formula>WEEKDAY(R$2)=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y22:AD22">
+    <cfRule type="expression" dxfId="0" priority="7">
+      <formula>WEEKDAY(AF$2)=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -1165,6 +1385,7 @@
     <hyperlink ref="B20" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
     <hyperlink ref="B21" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
     <hyperlink ref="B22" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B23" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1183,7 +1404,7 @@
     <row r="1" spans="2:151" ht="13" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:151" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C2" s="5">
         <v>46222</v>
@@ -1635,27 +1856,30 @@
     </row>
     <row r="3" spans="2:151" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
+      </c>
+      <c r="D3" s="16">
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="2:151" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="2:151" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="2:151" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="2:151" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh product plan spreadsheet
</commit_message>
<xml_diff>
--- a/products/product_plan.xlsx
+++ b/products/product_plan.xlsx
@@ -1,90 +1,203 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longtran/codes/bplatform/platform-ecosystem-docs/products/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C8491A-2CD4-3D41-821B-3768BEC93346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resource" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Overview" sheetId="1" r:id="rId1"/>
+    <sheet name="Resource" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+  <si>
+    <t>Project / Feature</t>
+  </si>
+  <si>
+    <t>MDFoods</t>
+  </si>
+  <si>
+    <t>◆ v1: User can see all products/contents</t>
+  </si>
+  <si>
+    <t>◆ v2: User can request a quote</t>
+  </si>
+  <si>
+    <t>◆ v3: User can complete an order</t>
+  </si>
+  <si>
+    <t>F-01: Master Layout</t>
+  </si>
+  <si>
+    <t>F-02: Landing Page (Home Page)</t>
+  </si>
+  <si>
+    <t>F-03: Product List by Category</t>
+  </si>
+  <si>
+    <t>F-04: Product Detail</t>
+  </si>
+  <si>
+    <t>F-05: Product Search</t>
+  </si>
+  <si>
+    <t>F-06: Static Pages</t>
+  </si>
+  <si>
+    <t>F-07: Activities</t>
+  </si>
+  <si>
+    <t>F-08: Registration</t>
+  </si>
+  <si>
+    <t>F-09: Authentication</t>
+  </si>
+  <si>
+    <t>F-10: Profile Management</t>
+  </si>
+  <si>
+    <t>F-11: Addresses Management</t>
+  </si>
+  <si>
+    <t>F-12: Company Information Management</t>
+  </si>
+  <si>
+    <t>F-13: Company Member/Permission Management</t>
+  </si>
+  <si>
+    <t>F-14: Shopping Cart</t>
+  </si>
+  <si>
+    <t>F-15: Request Quote Process</t>
+  </si>
+  <si>
+    <t>F-16: Quote Management</t>
+  </si>
+  <si>
+    <t>F-17: Order &amp; Payment</t>
+  </si>
+  <si>
+    <t>F-18: Orders Management</t>
+  </si>
+  <si>
+    <t>F-19: In-App Messages and Notification</t>
+  </si>
+  <si>
+    <t>F-20: Password Recovery</t>
+  </si>
+  <si>
+    <t>CRM</t>
+  </si>
+  <si>
+    <t>Odeli</t>
+  </si>
+  <si>
+    <t>LFarm</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>An Nguyen 1</t>
+  </si>
+  <si>
+    <t>Khuong Nguyen 1</t>
+  </si>
+  <si>
+    <t>Phat Phan 1</t>
+  </si>
+  <si>
+    <t>Phat Phan 2</t>
+  </si>
+  <si>
+    <t>Phat Ngo 1</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <color theme="0"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="9" tint="-0.249977111117893"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="9" tint="-0.249977111117893"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="10"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF9C5700"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color rgb="FF9C5700"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.0499893185216834"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.1499984740745262"/>
+        <fgColor theme="1" tint="0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.5999938962981048"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -161,163 +274,103 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.5999633777886288"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -637,1304 +690,1242 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:EU30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelRow="1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelRow="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="2.6640625" customWidth="1" min="1" max="1"/>
-    <col width="43.1640625" customWidth="1" min="2" max="2"/>
-    <col width="5.83203125" customWidth="1" style="2" min="3" max="3"/>
-    <col width="7.83203125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="5.83203125" bestFit="1" customWidth="1" min="5" max="151"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="43.1640625" customWidth="1"/>
+    <col min="3" max="3" width="5.83203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="151" width="5.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Project / Feature</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="n">
+    <row r="2" spans="2:151" x14ac:dyDescent="0.2">
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5">
         <v>46222</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="5">
         <v>46223</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="5">
         <v>46224</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="5">
         <v>46225</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="5">
         <v>46226</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="5">
         <v>46227</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="5">
         <v>46228</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="5">
         <v>46229</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="5">
         <v>46230</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="5">
         <v>46231</v>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="M2" s="5">
         <v>46232</v>
       </c>
-      <c r="N2" s="5" t="n">
+      <c r="N2" s="5">
         <v>46233</v>
       </c>
-      <c r="O2" s="5" t="n">
+      <c r="O2" s="5">
         <v>46234</v>
       </c>
-      <c r="P2" s="5" t="n">
+      <c r="P2" s="5">
         <v>46235</v>
       </c>
-      <c r="Q2" s="5" t="n">
+      <c r="Q2" s="5">
         <v>46236</v>
       </c>
-      <c r="R2" s="5" t="n">
+      <c r="R2" s="5">
         <v>46237</v>
       </c>
-      <c r="S2" s="5" t="n">
+      <c r="S2" s="5">
         <v>46238</v>
       </c>
-      <c r="T2" s="5" t="n">
+      <c r="T2" s="5">
         <v>46239</v>
       </c>
-      <c r="U2" s="5" t="n">
+      <c r="U2" s="5">
         <v>46240</v>
       </c>
-      <c r="V2" s="5" t="n">
+      <c r="V2" s="5">
         <v>46241</v>
       </c>
-      <c r="W2" s="5" t="n">
+      <c r="W2" s="5">
         <v>46242</v>
       </c>
-      <c r="X2" s="5" t="n">
+      <c r="X2" s="5">
         <v>46243</v>
       </c>
-      <c r="Y2" s="5" t="n">
+      <c r="Y2" s="5">
         <v>46244</v>
       </c>
-      <c r="Z2" s="5" t="n">
+      <c r="Z2" s="5">
         <v>46245</v>
       </c>
-      <c r="AA2" s="5" t="n">
+      <c r="AA2" s="5">
         <v>46246</v>
       </c>
-      <c r="AB2" s="5" t="n">
+      <c r="AB2" s="5">
         <v>46247</v>
       </c>
-      <c r="AC2" s="5" t="n">
+      <c r="AC2" s="5">
         <v>46248</v>
       </c>
-      <c r="AD2" s="5" t="n">
+      <c r="AD2" s="5">
         <v>46249</v>
       </c>
-      <c r="AE2" s="5" t="n">
+      <c r="AE2" s="5">
         <v>46250</v>
       </c>
-      <c r="AF2" s="5" t="n">
+      <c r="AF2" s="5">
         <v>46251</v>
       </c>
-      <c r="AG2" s="5" t="n">
+      <c r="AG2" s="5">
         <v>46252</v>
       </c>
-      <c r="AH2" s="5" t="n">
+      <c r="AH2" s="5">
         <v>46253</v>
       </c>
-      <c r="AI2" s="5" t="n">
+      <c r="AI2" s="5">
         <v>46254</v>
       </c>
-      <c r="AJ2" s="5" t="n">
+      <c r="AJ2" s="5">
         <v>46255</v>
       </c>
-      <c r="AK2" s="5" t="n">
+      <c r="AK2" s="5">
         <v>46256</v>
       </c>
-      <c r="AL2" s="5" t="n">
+      <c r="AL2" s="5">
         <v>46257</v>
       </c>
-      <c r="AM2" s="5" t="n">
+      <c r="AM2" s="5">
         <v>46258</v>
       </c>
-      <c r="AN2" s="5" t="n">
+      <c r="AN2" s="5">
         <v>46259</v>
       </c>
-      <c r="AO2" s="5" t="n">
+      <c r="AO2" s="5">
         <v>46260</v>
       </c>
-      <c r="AP2" s="5" t="n">
+      <c r="AP2" s="5">
         <v>46261</v>
       </c>
-      <c r="AQ2" s="5" t="n">
+      <c r="AQ2" s="5">
         <v>46262</v>
       </c>
-      <c r="AR2" s="5" t="n">
+      <c r="AR2" s="5">
         <v>46263</v>
       </c>
-      <c r="AS2" s="5" t="n">
+      <c r="AS2" s="5">
         <v>46264</v>
       </c>
-      <c r="AT2" s="5" t="n">
+      <c r="AT2" s="5">
         <v>46265</v>
       </c>
-      <c r="AU2" s="5" t="n">
+      <c r="AU2" s="5">
         <v>46266</v>
       </c>
-      <c r="AV2" s="5" t="n">
+      <c r="AV2" s="5">
         <v>46267</v>
       </c>
-      <c r="AW2" s="5" t="n">
+      <c r="AW2" s="5">
         <v>46268</v>
       </c>
-      <c r="AX2" s="5" t="n">
+      <c r="AX2" s="5">
         <v>46269</v>
       </c>
-      <c r="AY2" s="5" t="n">
+      <c r="AY2" s="5">
         <v>46270</v>
       </c>
-      <c r="AZ2" s="5" t="n">
+      <c r="AZ2" s="5">
         <v>46271</v>
       </c>
-      <c r="BA2" s="5" t="n">
+      <c r="BA2" s="5">
         <v>46272</v>
       </c>
-      <c r="BB2" s="5" t="n">
+      <c r="BB2" s="5">
         <v>46273</v>
       </c>
-      <c r="BC2" s="5" t="n">
+      <c r="BC2" s="5">
         <v>46274</v>
       </c>
-      <c r="BD2" s="5" t="n">
+      <c r="BD2" s="5">
         <v>46275</v>
       </c>
-      <c r="BE2" s="5" t="n">
+      <c r="BE2" s="5">
         <v>46276</v>
       </c>
-      <c r="BF2" s="5" t="n">
+      <c r="BF2" s="5">
         <v>46277</v>
       </c>
-      <c r="BG2" s="5" t="n">
+      <c r="BG2" s="5">
         <v>46278</v>
       </c>
-      <c r="BH2" s="5" t="n">
+      <c r="BH2" s="5">
         <v>46279</v>
       </c>
-      <c r="BI2" s="5" t="n">
+      <c r="BI2" s="5">
         <v>46280</v>
       </c>
-      <c r="BJ2" s="5" t="n">
+      <c r="BJ2" s="5">
         <v>46281</v>
       </c>
-      <c r="BK2" s="5" t="n">
+      <c r="BK2" s="5">
         <v>46282</v>
       </c>
-      <c r="BL2" s="5" t="n">
+      <c r="BL2" s="5">
         <v>46283</v>
       </c>
-      <c r="BM2" s="5" t="n">
+      <c r="BM2" s="5">
         <v>46284</v>
       </c>
-      <c r="BN2" s="5" t="n">
+      <c r="BN2" s="5">
         <v>46285</v>
       </c>
-      <c r="BO2" s="5" t="n">
+      <c r="BO2" s="5">
         <v>46286</v>
       </c>
-      <c r="BP2" s="5" t="n">
+      <c r="BP2" s="5">
         <v>46287</v>
       </c>
-      <c r="BQ2" s="5" t="n">
+      <c r="BQ2" s="5">
         <v>46288</v>
       </c>
-      <c r="BR2" s="5" t="n">
+      <c r="BR2" s="5">
         <v>46289</v>
       </c>
-      <c r="BS2" s="5" t="n">
+      <c r="BS2" s="5">
         <v>46290</v>
       </c>
-      <c r="BT2" s="5" t="n">
+      <c r="BT2" s="5">
         <v>46291</v>
       </c>
-      <c r="BU2" s="5" t="n">
+      <c r="BU2" s="5">
         <v>46292</v>
       </c>
-      <c r="BV2" s="5" t="n">
+      <c r="BV2" s="5">
         <v>46293</v>
       </c>
-      <c r="BW2" s="5" t="n">
+      <c r="BW2" s="5">
         <v>46294</v>
       </c>
-      <c r="BX2" s="5" t="n">
+      <c r="BX2" s="5">
         <v>46295</v>
       </c>
-      <c r="BY2" s="5" t="n">
+      <c r="BY2" s="5">
         <v>46296</v>
       </c>
-      <c r="BZ2" s="5" t="n">
+      <c r="BZ2" s="5">
         <v>46297</v>
       </c>
-      <c r="CA2" s="5" t="n">
+      <c r="CA2" s="5">
         <v>46298</v>
       </c>
-      <c r="CB2" s="5" t="n">
+      <c r="CB2" s="5">
         <v>46299</v>
       </c>
-      <c r="CC2" s="5" t="n">
+      <c r="CC2" s="5">
         <v>46300</v>
       </c>
-      <c r="CD2" s="5" t="n">
+      <c r="CD2" s="5">
         <v>46301</v>
       </c>
-      <c r="CE2" s="5" t="n">
+      <c r="CE2" s="5">
         <v>46302</v>
       </c>
-      <c r="CF2" s="5" t="n">
+      <c r="CF2" s="5">
         <v>46303</v>
       </c>
-      <c r="CG2" s="5" t="n">
+      <c r="CG2" s="5">
         <v>46304</v>
       </c>
-      <c r="CH2" s="5" t="n">
+      <c r="CH2" s="5">
         <v>46305</v>
       </c>
-      <c r="CI2" s="5" t="n">
+      <c r="CI2" s="5">
         <v>46306</v>
       </c>
-      <c r="CJ2" s="5" t="n">
+      <c r="CJ2" s="5">
         <v>46307</v>
       </c>
-      <c r="CK2" s="5" t="n">
+      <c r="CK2" s="5">
         <v>46308</v>
       </c>
-      <c r="CL2" s="5" t="n">
+      <c r="CL2" s="5">
         <v>46309</v>
       </c>
-      <c r="CM2" s="5" t="n">
+      <c r="CM2" s="5">
         <v>46310</v>
       </c>
-      <c r="CN2" s="5" t="n">
+      <c r="CN2" s="5">
         <v>46311</v>
       </c>
-      <c r="CO2" s="5" t="n">
+      <c r="CO2" s="5">
         <v>46312</v>
       </c>
-      <c r="CP2" s="5" t="n">
+      <c r="CP2" s="5">
         <v>46313</v>
       </c>
-      <c r="CQ2" s="5" t="n">
+      <c r="CQ2" s="5">
         <v>46314</v>
       </c>
-      <c r="CR2" s="5" t="n">
+      <c r="CR2" s="5">
         <v>46315</v>
       </c>
-      <c r="CS2" s="5" t="n">
+      <c r="CS2" s="5">
         <v>46316</v>
       </c>
-      <c r="CT2" s="5" t="n">
+      <c r="CT2" s="5">
         <v>46317</v>
       </c>
-      <c r="CU2" s="5" t="n">
+      <c r="CU2" s="5">
         <v>46318</v>
       </c>
-      <c r="CV2" s="5" t="n">
+      <c r="CV2" s="5">
         <v>46319</v>
       </c>
-      <c r="CW2" s="5" t="n">
+      <c r="CW2" s="5">
         <v>46320</v>
       </c>
-      <c r="CX2" s="5" t="n">
+      <c r="CX2" s="5">
         <v>46321</v>
       </c>
-      <c r="CY2" s="5" t="n">
+      <c r="CY2" s="5">
         <v>46322</v>
       </c>
-      <c r="CZ2" s="5" t="n">
+      <c r="CZ2" s="5">
         <v>46323</v>
       </c>
-      <c r="DA2" s="5" t="n">
+      <c r="DA2" s="5">
         <v>46324</v>
       </c>
-      <c r="DB2" s="5" t="n">
+      <c r="DB2" s="5">
         <v>46325</v>
       </c>
-      <c r="DC2" s="5" t="n">
+      <c r="DC2" s="5">
         <v>46326</v>
       </c>
-      <c r="DD2" s="5" t="n">
+      <c r="DD2" s="5">
         <v>46327</v>
       </c>
-      <c r="DE2" s="5" t="n">
+      <c r="DE2" s="5">
         <v>46328</v>
       </c>
-      <c r="DF2" s="5" t="n">
+      <c r="DF2" s="5">
         <v>46329</v>
       </c>
-      <c r="DG2" s="5" t="n">
+      <c r="DG2" s="5">
         <v>46330</v>
       </c>
-      <c r="DH2" s="5" t="n">
+      <c r="DH2" s="5">
         <v>46331</v>
       </c>
-      <c r="DI2" s="5" t="n">
+      <c r="DI2" s="5">
         <v>46332</v>
       </c>
-      <c r="DJ2" s="5" t="n">
+      <c r="DJ2" s="5">
         <v>46333</v>
       </c>
-      <c r="DK2" s="5" t="n">
+      <c r="DK2" s="5">
         <v>46334</v>
       </c>
-      <c r="DL2" s="5" t="n">
+      <c r="DL2" s="5">
         <v>46335</v>
       </c>
-      <c r="DM2" s="5" t="n">
+      <c r="DM2" s="5">
         <v>46336</v>
       </c>
-      <c r="DN2" s="5" t="n">
+      <c r="DN2" s="5">
         <v>46337</v>
       </c>
-      <c r="DO2" s="5" t="n">
+      <c r="DO2" s="5">
         <v>46338</v>
       </c>
-      <c r="DP2" s="5" t="n">
+      <c r="DP2" s="5">
         <v>46339</v>
       </c>
-      <c r="DQ2" s="5" t="n">
+      <c r="DQ2" s="5">
         <v>46340</v>
       </c>
-      <c r="DR2" s="5" t="n">
+      <c r="DR2" s="5">
         <v>46341</v>
       </c>
-      <c r="DS2" s="5" t="n">
+      <c r="DS2" s="5">
         <v>46342</v>
       </c>
-      <c r="DT2" s="5" t="n">
+      <c r="DT2" s="5">
         <v>46343</v>
       </c>
-      <c r="DU2" s="5" t="n">
+      <c r="DU2" s="5">
         <v>46344</v>
       </c>
-      <c r="DV2" s="5" t="n">
+      <c r="DV2" s="5">
         <v>46345</v>
       </c>
-      <c r="DW2" s="5" t="n">
+      <c r="DW2" s="5">
         <v>46346</v>
       </c>
-      <c r="DX2" s="5" t="n">
+      <c r="DX2" s="5">
         <v>46347</v>
       </c>
-      <c r="DY2" s="5" t="n">
+      <c r="DY2" s="5">
         <v>46348</v>
       </c>
-      <c r="DZ2" s="5" t="n">
+      <c r="DZ2" s="5">
         <v>46349</v>
       </c>
-      <c r="EA2" s="5" t="n">
+      <c r="EA2" s="5">
         <v>46350</v>
       </c>
-      <c r="EB2" s="5" t="n">
+      <c r="EB2" s="5">
         <v>46351</v>
       </c>
-      <c r="EC2" s="5" t="n">
+      <c r="EC2" s="5">
         <v>46352</v>
       </c>
-      <c r="ED2" s="5" t="n">
+      <c r="ED2" s="5">
         <v>46353</v>
       </c>
-      <c r="EE2" s="5" t="n">
+      <c r="EE2" s="5">
         <v>46354</v>
       </c>
-      <c r="EF2" s="5" t="n">
+      <c r="EF2" s="5">
         <v>46355</v>
       </c>
-      <c r="EG2" s="5" t="n">
+      <c r="EG2" s="5">
         <v>46356</v>
       </c>
-      <c r="EH2" s="5" t="n">
+      <c r="EH2" s="5">
         <v>46357</v>
       </c>
-      <c r="EI2" s="5" t="n">
+      <c r="EI2" s="5">
         <v>46358</v>
       </c>
-      <c r="EJ2" s="5" t="n">
+      <c r="EJ2" s="5">
         <v>46359</v>
       </c>
-      <c r="EK2" s="5" t="n">
+      <c r="EK2" s="5">
         <v>46360</v>
       </c>
-      <c r="EL2" s="5" t="n">
+      <c r="EL2" s="5">
         <v>46361</v>
       </c>
-      <c r="EM2" s="5" t="n">
+      <c r="EM2" s="5">
         <v>46362</v>
       </c>
-      <c r="EN2" s="5" t="n">
+      <c r="EN2" s="5">
         <v>46363</v>
       </c>
-      <c r="EO2" s="5" t="n">
+      <c r="EO2" s="5">
         <v>46364</v>
       </c>
-      <c r="EP2" s="5" t="n">
+      <c r="EP2" s="5">
         <v>46365</v>
       </c>
-      <c r="EQ2" s="5" t="n">
+      <c r="EQ2" s="5">
         <v>46366</v>
       </c>
-      <c r="ER2" s="5" t="n">
+      <c r="ER2" s="5">
         <v>46367</v>
       </c>
-      <c r="ES2" s="5" t="n">
+      <c r="ES2" s="5">
         <v>46368</v>
       </c>
-      <c r="ET2" s="5" t="n">
+      <c r="ET2" s="5">
         <v>46369</v>
       </c>
-      <c r="EU2" s="5" t="n">
+      <c r="EU2" s="5">
         <v>46370</v>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>MDFoods</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>◆ v1: User can see all products/contents</t>
-        </is>
-      </c>
-      <c r="X3" s="9" t="inlineStr">
-        <is>
-          <t>◆ v2: User can request a quote</t>
-        </is>
-      </c>
-      <c r="AE3" s="9" t="inlineStr">
-        <is>
-          <t>◆ v3: User can complete an order</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" outlineLevel="1">
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>F-01: Master Layout</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-    </row>
-    <row r="5" outlineLevel="1">
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>F-02: Landing Page (Home Page)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" outlineLevel="1">
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>F-03: Product List by Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" outlineLevel="1">
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>F-04: Product Detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" outlineLevel="1">
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>F-05: Product Search</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" outlineLevel="1">
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>F-06: Static Pages</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" outlineLevel="1">
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>F-07: Activities</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" outlineLevel="1">
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>F-08: Registration</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
-      <c r="H11" s="11" t="n"/>
-      <c r="I11" s="12" t="n"/>
-      <c r="K11" s="14" t="n"/>
-    </row>
-    <row r="12" outlineLevel="1">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>F-09: Authentication</t>
-        </is>
-      </c>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="K12" s="10" t="n"/>
-      <c r="L12" s="12" t="n"/>
-    </row>
-    <row r="13" outlineLevel="1">
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>F-10: Profile Management</t>
-        </is>
-      </c>
-      <c r="M13" s="10" t="n"/>
-      <c r="N13" s="11" t="n"/>
-      <c r="O13" s="12" t="n"/>
-    </row>
-    <row r="14" outlineLevel="1">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>F-11: Addresses Management</t>
-        </is>
-      </c>
-      <c r="M14" s="10" t="n"/>
-      <c r="N14" s="12" t="n"/>
-    </row>
-    <row r="15" outlineLevel="1">
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>F-12: Company Information Management</t>
-        </is>
-      </c>
-      <c r="O15" s="10" t="n"/>
-      <c r="P15" s="11" t="n"/>
-      <c r="R15" s="10" t="n"/>
-      <c r="S15" s="12" t="n"/>
-    </row>
-    <row r="16" outlineLevel="1">
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>F-13: Company Member/Permission Management</t>
-        </is>
-      </c>
-      <c r="T16" s="10" t="n"/>
-      <c r="U16" s="11" t="n"/>
-      <c r="V16" s="11" t="n"/>
-      <c r="W16" s="12" t="n"/>
-      <c r="Y16" s="14" t="n"/>
-    </row>
-    <row r="17" outlineLevel="1">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>F-14: Shopping Cart</t>
-        </is>
-      </c>
-      <c r="M17" s="10" t="n"/>
-      <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
-      <c r="R17" s="10" t="n"/>
-      <c r="S17" s="12" t="n"/>
-    </row>
-    <row r="18" outlineLevel="1">
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>F-15: Request Quote Process</t>
-        </is>
-      </c>
-      <c r="T18" s="10" t="n"/>
-      <c r="U18" s="12" t="n"/>
-    </row>
-    <row r="19" outlineLevel="1">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>F-16: Quote Management</t>
-        </is>
-      </c>
-      <c r="U19" s="10" t="n"/>
-      <c r="V19" s="11" t="n"/>
-      <c r="W19" s="12" t="n"/>
-    </row>
-    <row r="20" outlineLevel="1">
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>F-17: Order &amp; Payment</t>
-        </is>
-      </c>
-      <c r="Z20" s="10" t="n"/>
-      <c r="AA20" s="11" t="n"/>
-      <c r="AB20" s="11" t="n"/>
-      <c r="AC20" s="11" t="n"/>
-      <c r="AD20" s="12" t="n"/>
-    </row>
-    <row r="21" outlineLevel="1">
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>F-18: Orders Management</t>
-        </is>
-      </c>
-      <c r="Z21" s="10" t="n"/>
-      <c r="AA21" s="12" t="n"/>
-    </row>
-    <row r="22" outlineLevel="1">
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>F-19: In-App Messages and Notification</t>
-        </is>
-      </c>
-      <c r="Z22" s="10" t="n"/>
-      <c r="AA22" s="11" t="n"/>
-      <c r="AB22" s="11" t="n"/>
-      <c r="AC22" s="11" t="n"/>
-      <c r="AD22" s="11" t="n"/>
-      <c r="AF22" s="14" t="n"/>
-    </row>
-    <row r="23" outlineLevel="1">
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>F-20: Password Recovery</t>
-        </is>
-      </c>
-      <c r="M23" s="10" t="n"/>
-      <c r="N23" s="11" t="n"/>
-      <c r="O23" s="12" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>CRM</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="7" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>Odeli</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="7" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="1" t="inlineStr">
-        <is>
-          <t>LFarm</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="7" t="n"/>
+    <row r="3" spans="2:151" x14ac:dyDescent="0.2">
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE3" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="12"/>
+      <c r="K11" s="13"/>
+    </row>
+    <row r="12" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="12"/>
+    </row>
+    <row r="13" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="M13" s="10"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="12"/>
+    </row>
+    <row r="14" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="M14" s="10"/>
+      <c r="N14" s="12"/>
+    </row>
+    <row r="15" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="O15" s="10"/>
+      <c r="P15" s="11"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="12"/>
+    </row>
+    <row r="16" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="T16" s="10"/>
+      <c r="U16" s="11"/>
+      <c r="V16" s="11"/>
+      <c r="W16" s="12"/>
+      <c r="Y16" s="13"/>
+    </row>
+    <row r="17" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="M17" s="10"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="11"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="12"/>
+    </row>
+    <row r="18" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="T18" s="10"/>
+      <c r="U18" s="12"/>
+    </row>
+    <row r="19" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="U19" s="10"/>
+      <c r="V19" s="11"/>
+      <c r="W19" s="12"/>
+    </row>
+    <row r="20" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="Z20" s="10"/>
+      <c r="AA20" s="11"/>
+      <c r="AB20" s="11"/>
+      <c r="AC20" s="11"/>
+      <c r="AD20" s="12"/>
+    </row>
+    <row r="21" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z21" s="10"/>
+      <c r="AA21" s="12"/>
+    </row>
+    <row r="22" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z22" s="10"/>
+      <c r="AA22" s="11"/>
+      <c r="AB22" s="11"/>
+      <c r="AC22" s="11"/>
+      <c r="AD22" s="11"/>
+      <c r="AF22" s="13"/>
+    </row>
+    <row r="23" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M23" s="10"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="12"/>
+    </row>
+    <row r="25" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="6"/>
+    </row>
+    <row r="26" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B26" s="7"/>
+    </row>
+    <row r="27" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="6"/>
+    </row>
+    <row r="28" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B28" s="7"/>
+    </row>
+    <row r="29" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="6"/>
+    </row>
+    <row r="30" spans="2:32" x14ac:dyDescent="0.2">
+      <c r="B30" s="7"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:EU10 C11:C12 C13:J23 C24:P26 C27:EU1048576 J11:EU12 Q13:Q26 R17:W17 R24:EU26 S13:EU14 S20:X22 S23:EU23 V15:EU15 V18:EU18 X16:EU17 X19:EU19 AE20:AE22 AF20:EU21 AL22:EU22">
-    <cfRule type="expression" priority="3" dxfId="0">
+  <conditionalFormatting sqref="C2:EU10 C11:C12 J11:EU12 S13:EU14 C13:J23 Q13:Q26 V15:EU15 X16:EU17 R17:W17 V18:EU18 X19:EU19 AF20:EU21 S20:X22 AE20:AE22 AL22:EU22 S23:EU23 C24:P26 R24:EU26 C27:EU1048576">
+    <cfRule type="expression" dxfId="7" priority="3">
       <formula>WEEKDAY(C$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E11:I11 T16:W16 T18:U18 Z20:AD21">
+    <cfRule type="expression" dxfId="6" priority="11">
+      <formula>WEEKDAY(D$2)=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F12:I12 M13:P14 R13:R14 M15:N15 R16 M16:P23 R18:R23">
+    <cfRule type="expression" dxfId="5" priority="13">
+      <formula>WEEKDAY(D$2)=1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="O15:P15">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>WEEKDAY(R$2)=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R15:S15">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>WEEKDAY(R$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U19:W19">
-    <cfRule type="expression" priority="7" dxfId="0">
+    <cfRule type="expression" dxfId="2" priority="7">
       <formula>WEEKDAY(R$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z22:AD22">
-    <cfRule type="expression" priority="9" dxfId="0">
+    <cfRule type="expression" dxfId="1" priority="9">
       <formula>WEEKDAY(AF$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E11:I11 T16:W16 T18:U18 Z20:AD21">
-    <cfRule type="expression" priority="11" dxfId="0">
-      <formula>WEEKDAY(D$2)=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F12:I12 M13:P14 M15:N15 M16:P23 R13:R14 R16 R18:R23">
-    <cfRule type="expression" priority="13" dxfId="0">
-      <formula>WEEKDAY(D$2)=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R15:S15">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>WEEKDAY(R$2)=1</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="AF22">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>WEEKDAY(AF$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId20"/>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="B7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="B8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="B9" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B10" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B11" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="B12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="B13" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="B14" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="B15" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="B16" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="B17" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="B18" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="B19" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="B20" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="B21" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B22" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B23" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:EU7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="2.6640625" customWidth="1" min="1" max="1"/>
-    <col width="18.83203125" customWidth="1" min="2" max="2"/>
-    <col width="5.83203125" bestFit="1" customWidth="1" min="3" max="151"/>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="151" width="5.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13" customHeight="1"/>
-    <row r="2" customFormat="1" s="3">
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="n">
+    <row r="1" spans="1:151" ht="13" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:151" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="5">
         <v>46222</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="5">
         <v>46223</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="5">
         <v>46224</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="5">
         <v>46225</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="5">
         <v>46226</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="5">
         <v>46227</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="5">
         <v>46228</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="5">
         <v>46229</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="5">
         <v>46230</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="5">
         <v>46231</v>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="M2" s="5">
         <v>46232</v>
       </c>
-      <c r="N2" s="5" t="n">
+      <c r="N2" s="5">
         <v>46233</v>
       </c>
-      <c r="O2" s="5" t="n">
+      <c r="O2" s="5">
         <v>46234</v>
       </c>
-      <c r="P2" s="5" t="n">
+      <c r="P2" s="5">
         <v>46235</v>
       </c>
-      <c r="Q2" s="5" t="n">
+      <c r="Q2" s="5">
         <v>46236</v>
       </c>
-      <c r="R2" s="5" t="n">
+      <c r="R2" s="5">
         <v>46237</v>
       </c>
-      <c r="S2" s="5" t="n">
+      <c r="S2" s="5">
         <v>46238</v>
       </c>
-      <c r="T2" s="5" t="n">
+      <c r="T2" s="5">
         <v>46239</v>
       </c>
-      <c r="U2" s="5" t="n">
+      <c r="U2" s="5">
         <v>46240</v>
       </c>
-      <c r="V2" s="5" t="n">
+      <c r="V2" s="5">
         <v>46241</v>
       </c>
-      <c r="W2" s="5" t="n">
+      <c r="W2" s="5">
         <v>46242</v>
       </c>
-      <c r="X2" s="5" t="n">
+      <c r="X2" s="5">
         <v>46243</v>
       </c>
-      <c r="Y2" s="5" t="n">
+      <c r="Y2" s="5">
         <v>46244</v>
       </c>
-      <c r="Z2" s="5" t="n">
+      <c r="Z2" s="5">
         <v>46245</v>
       </c>
-      <c r="AA2" s="5" t="n">
+      <c r="AA2" s="5">
         <v>46246</v>
       </c>
-      <c r="AB2" s="5" t="n">
+      <c r="AB2" s="5">
         <v>46247</v>
       </c>
-      <c r="AC2" s="5" t="n">
+      <c r="AC2" s="5">
         <v>46248</v>
       </c>
-      <c r="AD2" s="5" t="n">
+      <c r="AD2" s="5">
         <v>46249</v>
       </c>
-      <c r="AE2" s="5" t="n">
+      <c r="AE2" s="5">
         <v>46250</v>
       </c>
-      <c r="AF2" s="5" t="n">
+      <c r="AF2" s="5">
         <v>46251</v>
       </c>
-      <c r="AG2" s="5" t="n">
+      <c r="AG2" s="5">
         <v>46252</v>
       </c>
-      <c r="AH2" s="5" t="n">
+      <c r="AH2" s="5">
         <v>46253</v>
       </c>
-      <c r="AI2" s="5" t="n">
+      <c r="AI2" s="5">
         <v>46254</v>
       </c>
-      <c r="AJ2" s="5" t="n">
+      <c r="AJ2" s="5">
         <v>46255</v>
       </c>
-      <c r="AK2" s="5" t="n">
+      <c r="AK2" s="5">
         <v>46256</v>
       </c>
-      <c r="AL2" s="5" t="n">
+      <c r="AL2" s="5">
         <v>46257</v>
       </c>
-      <c r="AM2" s="5" t="n">
+      <c r="AM2" s="5">
         <v>46258</v>
       </c>
-      <c r="AN2" s="5" t="n">
+      <c r="AN2" s="5">
         <v>46259</v>
       </c>
-      <c r="AO2" s="5" t="n">
+      <c r="AO2" s="5">
         <v>46260</v>
       </c>
-      <c r="AP2" s="5" t="n">
+      <c r="AP2" s="5">
         <v>46261</v>
       </c>
-      <c r="AQ2" s="5" t="n">
+      <c r="AQ2" s="5">
         <v>46262</v>
       </c>
-      <c r="AR2" s="5" t="n">
+      <c r="AR2" s="5">
         <v>46263</v>
       </c>
-      <c r="AS2" s="5" t="n">
+      <c r="AS2" s="5">
         <v>46264</v>
       </c>
-      <c r="AT2" s="5" t="n">
+      <c r="AT2" s="5">
         <v>46265</v>
       </c>
-      <c r="AU2" s="5" t="n">
+      <c r="AU2" s="5">
         <v>46266</v>
       </c>
-      <c r="AV2" s="5" t="n">
+      <c r="AV2" s="5">
         <v>46267</v>
       </c>
-      <c r="AW2" s="5" t="n">
+      <c r="AW2" s="5">
         <v>46268</v>
       </c>
-      <c r="AX2" s="5" t="n">
+      <c r="AX2" s="5">
         <v>46269</v>
       </c>
-      <c r="AY2" s="5" t="n">
+      <c r="AY2" s="5">
         <v>46270</v>
       </c>
-      <c r="AZ2" s="5" t="n">
+      <c r="AZ2" s="5">
         <v>46271</v>
       </c>
-      <c r="BA2" s="5" t="n">
+      <c r="BA2" s="5">
         <v>46272</v>
       </c>
-      <c r="BB2" s="5" t="n">
+      <c r="BB2" s="5">
         <v>46273</v>
       </c>
-      <c r="BC2" s="5" t="n">
+      <c r="BC2" s="5">
         <v>46274</v>
       </c>
-      <c r="BD2" s="5" t="n">
+      <c r="BD2" s="5">
         <v>46275</v>
       </c>
-      <c r="BE2" s="5" t="n">
+      <c r="BE2" s="5">
         <v>46276</v>
       </c>
-      <c r="BF2" s="5" t="n">
+      <c r="BF2" s="5">
         <v>46277</v>
       </c>
-      <c r="BG2" s="5" t="n">
+      <c r="BG2" s="5">
         <v>46278</v>
       </c>
-      <c r="BH2" s="5" t="n">
+      <c r="BH2" s="5">
         <v>46279</v>
       </c>
-      <c r="BI2" s="5" t="n">
+      <c r="BI2" s="5">
         <v>46280</v>
       </c>
-      <c r="BJ2" s="5" t="n">
+      <c r="BJ2" s="5">
         <v>46281</v>
       </c>
-      <c r="BK2" s="5" t="n">
+      <c r="BK2" s="5">
         <v>46282</v>
       </c>
-      <c r="BL2" s="5" t="n">
+      <c r="BL2" s="5">
         <v>46283</v>
       </c>
-      <c r="BM2" s="5" t="n">
+      <c r="BM2" s="5">
         <v>46284</v>
       </c>
-      <c r="BN2" s="5" t="n">
+      <c r="BN2" s="5">
         <v>46285</v>
       </c>
-      <c r="BO2" s="5" t="n">
+      <c r="BO2" s="5">
         <v>46286</v>
       </c>
-      <c r="BP2" s="5" t="n">
+      <c r="BP2" s="5">
         <v>46287</v>
       </c>
-      <c r="BQ2" s="5" t="n">
+      <c r="BQ2" s="5">
         <v>46288</v>
       </c>
-      <c r="BR2" s="5" t="n">
+      <c r="BR2" s="5">
         <v>46289</v>
       </c>
-      <c r="BS2" s="5" t="n">
+      <c r="BS2" s="5">
         <v>46290</v>
       </c>
-      <c r="BT2" s="5" t="n">
+      <c r="BT2" s="5">
         <v>46291</v>
       </c>
-      <c r="BU2" s="5" t="n">
+      <c r="BU2" s="5">
         <v>46292</v>
       </c>
-      <c r="BV2" s="5" t="n">
+      <c r="BV2" s="5">
         <v>46293</v>
       </c>
-      <c r="BW2" s="5" t="n">
+      <c r="BW2" s="5">
         <v>46294</v>
       </c>
-      <c r="BX2" s="5" t="n">
+      <c r="BX2" s="5">
         <v>46295</v>
       </c>
-      <c r="BY2" s="5" t="n">
+      <c r="BY2" s="5">
         <v>46296</v>
       </c>
-      <c r="BZ2" s="5" t="n">
+      <c r="BZ2" s="5">
         <v>46297</v>
       </c>
-      <c r="CA2" s="5" t="n">
+      <c r="CA2" s="5">
         <v>46298</v>
       </c>
-      <c r="CB2" s="5" t="n">
+      <c r="CB2" s="5">
         <v>46299</v>
       </c>
-      <c r="CC2" s="5" t="n">
+      <c r="CC2" s="5">
         <v>46300</v>
       </c>
-      <c r="CD2" s="5" t="n">
+      <c r="CD2" s="5">
         <v>46301</v>
       </c>
-      <c r="CE2" s="5" t="n">
+      <c r="CE2" s="5">
         <v>46302</v>
       </c>
-      <c r="CF2" s="5" t="n">
+      <c r="CF2" s="5">
         <v>46303</v>
       </c>
-      <c r="CG2" s="5" t="n">
+      <c r="CG2" s="5">
         <v>46304</v>
       </c>
-      <c r="CH2" s="5" t="n">
+      <c r="CH2" s="5">
         <v>46305</v>
       </c>
-      <c r="CI2" s="5" t="n">
+      <c r="CI2" s="5">
         <v>46306</v>
       </c>
-      <c r="CJ2" s="5" t="n">
+      <c r="CJ2" s="5">
         <v>46307</v>
       </c>
-      <c r="CK2" s="5" t="n">
+      <c r="CK2" s="5">
         <v>46308</v>
       </c>
-      <c r="CL2" s="5" t="n">
+      <c r="CL2" s="5">
         <v>46309</v>
       </c>
-      <c r="CM2" s="5" t="n">
+      <c r="CM2" s="5">
         <v>46310</v>
       </c>
-      <c r="CN2" s="5" t="n">
+      <c r="CN2" s="5">
         <v>46311</v>
       </c>
-      <c r="CO2" s="5" t="n">
+      <c r="CO2" s="5">
         <v>46312</v>
       </c>
-      <c r="CP2" s="5" t="n">
+      <c r="CP2" s="5">
         <v>46313</v>
       </c>
-      <c r="CQ2" s="5" t="n">
+      <c r="CQ2" s="5">
         <v>46314</v>
       </c>
-      <c r="CR2" s="5" t="n">
+      <c r="CR2" s="5">
         <v>46315</v>
       </c>
-      <c r="CS2" s="5" t="n">
+      <c r="CS2" s="5">
         <v>46316</v>
       </c>
-      <c r="CT2" s="5" t="n">
+      <c r="CT2" s="5">
         <v>46317</v>
       </c>
-      <c r="CU2" s="5" t="n">
+      <c r="CU2" s="5">
         <v>46318</v>
       </c>
-      <c r="CV2" s="5" t="n">
+      <c r="CV2" s="5">
         <v>46319</v>
       </c>
-      <c r="CW2" s="5" t="n">
+      <c r="CW2" s="5">
         <v>46320</v>
       </c>
-      <c r="CX2" s="5" t="n">
+      <c r="CX2" s="5">
         <v>46321</v>
       </c>
-      <c r="CY2" s="5" t="n">
+      <c r="CY2" s="5">
         <v>46322</v>
       </c>
-      <c r="CZ2" s="5" t="n">
+      <c r="CZ2" s="5">
         <v>46323</v>
       </c>
-      <c r="DA2" s="5" t="n">
+      <c r="DA2" s="5">
         <v>46324</v>
       </c>
-      <c r="DB2" s="5" t="n">
+      <c r="DB2" s="5">
         <v>46325</v>
       </c>
-      <c r="DC2" s="5" t="n">
+      <c r="DC2" s="5">
         <v>46326</v>
       </c>
-      <c r="DD2" s="5" t="n">
+      <c r="DD2" s="5">
         <v>46327</v>
       </c>
-      <c r="DE2" s="5" t="n">
+      <c r="DE2" s="5">
         <v>46328</v>
       </c>
-      <c r="DF2" s="5" t="n">
+      <c r="DF2" s="5">
         <v>46329</v>
       </c>
-      <c r="DG2" s="5" t="n">
+      <c r="DG2" s="5">
         <v>46330</v>
       </c>
-      <c r="DH2" s="5" t="n">
+      <c r="DH2" s="5">
         <v>46331</v>
       </c>
-      <c r="DI2" s="5" t="n">
+      <c r="DI2" s="5">
         <v>46332</v>
       </c>
-      <c r="DJ2" s="5" t="n">
+      <c r="DJ2" s="5">
         <v>46333</v>
       </c>
-      <c r="DK2" s="5" t="n">
+      <c r="DK2" s="5">
         <v>46334</v>
       </c>
-      <c r="DL2" s="5" t="n">
+      <c r="DL2" s="5">
         <v>46335</v>
       </c>
-      <c r="DM2" s="5" t="n">
+      <c r="DM2" s="5">
         <v>46336</v>
       </c>
-      <c r="DN2" s="5" t="n">
+      <c r="DN2" s="5">
         <v>46337</v>
       </c>
-      <c r="DO2" s="5" t="n">
+      <c r="DO2" s="5">
         <v>46338</v>
       </c>
-      <c r="DP2" s="5" t="n">
+      <c r="DP2" s="5">
         <v>46339</v>
       </c>
-      <c r="DQ2" s="5" t="n">
+      <c r="DQ2" s="5">
         <v>46340</v>
       </c>
-      <c r="DR2" s="5" t="n">
+      <c r="DR2" s="5">
         <v>46341</v>
       </c>
-      <c r="DS2" s="5" t="n">
+      <c r="DS2" s="5">
         <v>46342</v>
       </c>
-      <c r="DT2" s="5" t="n">
+      <c r="DT2" s="5">
         <v>46343</v>
       </c>
-      <c r="DU2" s="5" t="n">
+      <c r="DU2" s="5">
         <v>46344</v>
       </c>
-      <c r="DV2" s="5" t="n">
+      <c r="DV2" s="5">
         <v>46345</v>
       </c>
-      <c r="DW2" s="5" t="n">
+      <c r="DW2" s="5">
         <v>46346</v>
       </c>
-      <c r="DX2" s="5" t="n">
+      <c r="DX2" s="5">
         <v>46347</v>
       </c>
-      <c r="DY2" s="5" t="n">
+      <c r="DY2" s="5">
         <v>46348</v>
       </c>
-      <c r="DZ2" s="5" t="n">
+      <c r="DZ2" s="5">
         <v>46349</v>
       </c>
-      <c r="EA2" s="5" t="n">
+      <c r="EA2" s="5">
         <v>46350</v>
       </c>
-      <c r="EB2" s="5" t="n">
+      <c r="EB2" s="5">
         <v>46351</v>
       </c>
-      <c r="EC2" s="5" t="n">
+      <c r="EC2" s="5">
         <v>46352</v>
       </c>
-      <c r="ED2" s="5" t="n">
+      <c r="ED2" s="5">
         <v>46353</v>
       </c>
-      <c r="EE2" s="5" t="n">
+      <c r="EE2" s="5">
         <v>46354</v>
       </c>
-      <c r="EF2" s="5" t="n">
+      <c r="EF2" s="5">
         <v>46355</v>
       </c>
-      <c r="EG2" s="5" t="n">
+      <c r="EG2" s="5">
         <v>46356</v>
       </c>
-      <c r="EH2" s="5" t="n">
+      <c r="EH2" s="5">
         <v>46357</v>
       </c>
-      <c r="EI2" s="5" t="n">
+      <c r="EI2" s="5">
         <v>46358</v>
       </c>
-      <c r="EJ2" s="5" t="n">
+      <c r="EJ2" s="5">
         <v>46359</v>
       </c>
-      <c r="EK2" s="5" t="n">
+      <c r="EK2" s="5">
         <v>46360</v>
       </c>
-      <c r="EL2" s="5" t="n">
+      <c r="EL2" s="5">
         <v>46361</v>
       </c>
-      <c r="EM2" s="5" t="n">
+      <c r="EM2" s="5">
         <v>46362</v>
       </c>
-      <c r="EN2" s="5" t="n">
+      <c r="EN2" s="5">
         <v>46363</v>
       </c>
-      <c r="EO2" s="5" t="n">
+      <c r="EO2" s="5">
         <v>46364</v>
       </c>
-      <c r="EP2" s="5" t="n">
+      <c r="EP2" s="5">
         <v>46365</v>
       </c>
-      <c r="EQ2" s="5" t="n">
+      <c r="EQ2" s="5">
         <v>46366</v>
       </c>
-      <c r="ER2" s="5" t="n">
+      <c r="ER2" s="5">
         <v>46367</v>
       </c>
-      <c r="ES2" s="5" t="n">
+      <c r="ES2" s="5">
         <v>46368</v>
       </c>
-      <c r="ET2" s="5" t="n">
+      <c r="ET2" s="5">
         <v>46369</v>
       </c>
-      <c r="EU2" s="5" t="n">
+      <c r="EU2" s="5">
         <v>46370</v>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>An Nguyen 1</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="n">
+    <row r="3" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3"/>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="15">
         <v>5</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="14">
         <v>8</v>
       </c>
     </row>
-    <row r="4">
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Khuong Nguyen 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Phat Phan 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Phat Phan 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Phat Ngo 1</t>
-        </is>
+    <row r="4" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4"/>
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5"/>
+      <c r="B5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6"/>
+      <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7"/>
+      <c r="B7" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update product docs and triage agent
</commit_message>
<xml_diff>
--- a/products/product_plan.xlsx
+++ b/products/product_plan.xlsx
@@ -1,203 +1,90 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longtran/codes/bplatform/platform-ecosystem-docs/products/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C8491A-2CD4-3D41-821B-3768BEC93346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" r:id="rId1"/>
-    <sheet name="Resource" sheetId="2" r:id="rId2"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resource" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
-  <si>
-    <t>Project / Feature</t>
-  </si>
-  <si>
-    <t>MDFoods</t>
-  </si>
-  <si>
-    <t>◆ v1: User can see all products/contents</t>
-  </si>
-  <si>
-    <t>◆ v2: User can request a quote</t>
-  </si>
-  <si>
-    <t>◆ v3: User can complete an order</t>
-  </si>
-  <si>
-    <t>F-01: Master Layout</t>
-  </si>
-  <si>
-    <t>F-02: Landing Page (Home Page)</t>
-  </si>
-  <si>
-    <t>F-03: Product List by Category</t>
-  </si>
-  <si>
-    <t>F-04: Product Detail</t>
-  </si>
-  <si>
-    <t>F-05: Product Search</t>
-  </si>
-  <si>
-    <t>F-06: Static Pages</t>
-  </si>
-  <si>
-    <t>F-07: Activities</t>
-  </si>
-  <si>
-    <t>F-08: Registration</t>
-  </si>
-  <si>
-    <t>F-09: Authentication</t>
-  </si>
-  <si>
-    <t>F-10: Profile Management</t>
-  </si>
-  <si>
-    <t>F-11: Addresses Management</t>
-  </si>
-  <si>
-    <t>F-12: Company Information Management</t>
-  </si>
-  <si>
-    <t>F-13: Company Member/Permission Management</t>
-  </si>
-  <si>
-    <t>F-14: Shopping Cart</t>
-  </si>
-  <si>
-    <t>F-15: Request Quote Process</t>
-  </si>
-  <si>
-    <t>F-16: Quote Management</t>
-  </si>
-  <si>
-    <t>F-17: Order &amp; Payment</t>
-  </si>
-  <si>
-    <t>F-18: Orders Management</t>
-  </si>
-  <si>
-    <t>F-19: In-App Messages and Notification</t>
-  </si>
-  <si>
-    <t>F-20: Password Recovery</t>
-  </si>
-  <si>
-    <t>CRM</t>
-  </si>
-  <si>
-    <t>Odeli</t>
-  </si>
-  <si>
-    <t>LFarm</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>An Nguyen 1</t>
-  </si>
-  <si>
-    <t>Khuong Nguyen 1</t>
-  </si>
-  <si>
-    <t>Phat Phan 1</t>
-  </si>
-  <si>
-    <t>Phat Phan 2</t>
-  </si>
-  <si>
-    <t>Phat Ngo 1</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="0"/>
       <sz val="12"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="9" tint="-0.249977111117893"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="9" tint="-0.249977111117893"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF9C5700"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color rgb="FF9C5700"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <fgColor theme="0" tint="-0.0499893185216834"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.14999847407452621"/>
+        <fgColor theme="1" tint="0.1499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -274,103 +161,163 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor theme="5" tint="0.5999633777886288"/>
         </patternFill>
       </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -690,1242 +637,1343 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:EU30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelRow="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="43.1640625" customWidth="1"/>
-    <col min="3" max="3" width="5.83203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="151" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col width="2.6640625" customWidth="1" style="14" min="1" max="1"/>
+    <col width="43.1640625" customWidth="1" style="14" min="2" max="2"/>
+    <col width="5.83203125" customWidth="1" style="2" min="3" max="3"/>
+    <col width="7.83203125" bestFit="1" customWidth="1" style="14" min="4" max="4"/>
+    <col width="5.83203125" bestFit="1" customWidth="1" style="14" min="5" max="151"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:151" x14ac:dyDescent="0.2">
-      <c r="B2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="5">
+    <row r="2">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Project / Feature</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>46222</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="5" t="n">
         <v>46223</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="5" t="n">
         <v>46224</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="5" t="n">
         <v>46225</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="5" t="n">
         <v>46226</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="5" t="n">
         <v>46227</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="5" t="n">
         <v>46228</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="5" t="n">
         <v>46229</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="5" t="n">
         <v>46230</v>
       </c>
-      <c r="L2" s="5">
+      <c r="L2" s="5" t="n">
         <v>46231</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2" s="5" t="n">
         <v>46232</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="5" t="n">
         <v>46233</v>
       </c>
-      <c r="O2" s="5">
+      <c r="O2" s="5" t="n">
         <v>46234</v>
       </c>
-      <c r="P2" s="5">
+      <c r="P2" s="5" t="n">
         <v>46235</v>
       </c>
-      <c r="Q2" s="5">
+      <c r="Q2" s="5" t="n">
         <v>46236</v>
       </c>
-      <c r="R2" s="5">
+      <c r="R2" s="5" t="n">
         <v>46237</v>
       </c>
-      <c r="S2" s="5">
+      <c r="S2" s="5" t="n">
         <v>46238</v>
       </c>
-      <c r="T2" s="5">
+      <c r="T2" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="U2" s="5">
+      <c r="U2" s="5" t="n">
         <v>46240</v>
       </c>
-      <c r="V2" s="5">
+      <c r="V2" s="5" t="n">
         <v>46241</v>
       </c>
-      <c r="W2" s="5">
+      <c r="W2" s="5" t="n">
         <v>46242</v>
       </c>
-      <c r="X2" s="5">
+      <c r="X2" s="5" t="n">
         <v>46243</v>
       </c>
-      <c r="Y2" s="5">
+      <c r="Y2" s="5" t="n">
         <v>46244</v>
       </c>
-      <c r="Z2" s="5">
+      <c r="Z2" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="AA2" s="5">
+      <c r="AA2" s="5" t="n">
         <v>46246</v>
       </c>
-      <c r="AB2" s="5">
+      <c r="AB2" s="5" t="n">
         <v>46247</v>
       </c>
-      <c r="AC2" s="5">
+      <c r="AC2" s="5" t="n">
         <v>46248</v>
       </c>
-      <c r="AD2" s="5">
+      <c r="AD2" s="5" t="n">
         <v>46249</v>
       </c>
-      <c r="AE2" s="5">
+      <c r="AE2" s="5" t="n">
         <v>46250</v>
       </c>
-      <c r="AF2" s="5">
+      <c r="AF2" s="5" t="n">
         <v>46251</v>
       </c>
-      <c r="AG2" s="5">
+      <c r="AG2" s="5" t="n">
         <v>46252</v>
       </c>
-      <c r="AH2" s="5">
+      <c r="AH2" s="5" t="n">
         <v>46253</v>
       </c>
-      <c r="AI2" s="5">
+      <c r="AI2" s="5" t="n">
         <v>46254</v>
       </c>
-      <c r="AJ2" s="5">
+      <c r="AJ2" s="5" t="n">
         <v>46255</v>
       </c>
-      <c r="AK2" s="5">
+      <c r="AK2" s="5" t="n">
         <v>46256</v>
       </c>
-      <c r="AL2" s="5">
+      <c r="AL2" s="5" t="n">
         <v>46257</v>
       </c>
-      <c r="AM2" s="5">
+      <c r="AM2" s="5" t="n">
         <v>46258</v>
       </c>
-      <c r="AN2" s="5">
+      <c r="AN2" s="5" t="n">
         <v>46259</v>
       </c>
-      <c r="AO2" s="5">
+      <c r="AO2" s="5" t="n">
         <v>46260</v>
       </c>
-      <c r="AP2" s="5">
+      <c r="AP2" s="5" t="n">
         <v>46261</v>
       </c>
-      <c r="AQ2" s="5">
+      <c r="AQ2" s="5" t="n">
         <v>46262</v>
       </c>
-      <c r="AR2" s="5">
+      <c r="AR2" s="5" t="n">
         <v>46263</v>
       </c>
-      <c r="AS2" s="5">
+      <c r="AS2" s="5" t="n">
         <v>46264</v>
       </c>
-      <c r="AT2" s="5">
+      <c r="AT2" s="5" t="n">
         <v>46265</v>
       </c>
-      <c r="AU2" s="5">
+      <c r="AU2" s="5" t="n">
         <v>46266</v>
       </c>
-      <c r="AV2" s="5">
+      <c r="AV2" s="5" t="n">
         <v>46267</v>
       </c>
-      <c r="AW2" s="5">
+      <c r="AW2" s="5" t="n">
         <v>46268</v>
       </c>
-      <c r="AX2" s="5">
+      <c r="AX2" s="5" t="n">
         <v>46269</v>
       </c>
-      <c r="AY2" s="5">
+      <c r="AY2" s="5" t="n">
         <v>46270</v>
       </c>
-      <c r="AZ2" s="5">
+      <c r="AZ2" s="5" t="n">
         <v>46271</v>
       </c>
-      <c r="BA2" s="5">
+      <c r="BA2" s="5" t="n">
         <v>46272</v>
       </c>
-      <c r="BB2" s="5">
+      <c r="BB2" s="5" t="n">
         <v>46273</v>
       </c>
-      <c r="BC2" s="5">
+      <c r="BC2" s="5" t="n">
         <v>46274</v>
       </c>
-      <c r="BD2" s="5">
+      <c r="BD2" s="5" t="n">
         <v>46275</v>
       </c>
-      <c r="BE2" s="5">
+      <c r="BE2" s="5" t="n">
         <v>46276</v>
       </c>
-      <c r="BF2" s="5">
+      <c r="BF2" s="5" t="n">
         <v>46277</v>
       </c>
-      <c r="BG2" s="5">
+      <c r="BG2" s="5" t="n">
         <v>46278</v>
       </c>
-      <c r="BH2" s="5">
+      <c r="BH2" s="5" t="n">
         <v>46279</v>
       </c>
-      <c r="BI2" s="5">
+      <c r="BI2" s="5" t="n">
         <v>46280</v>
       </c>
-      <c r="BJ2" s="5">
+      <c r="BJ2" s="5" t="n">
         <v>46281</v>
       </c>
-      <c r="BK2" s="5">
+      <c r="BK2" s="5" t="n">
         <v>46282</v>
       </c>
-      <c r="BL2" s="5">
+      <c r="BL2" s="5" t="n">
         <v>46283</v>
       </c>
-      <c r="BM2" s="5">
+      <c r="BM2" s="5" t="n">
         <v>46284</v>
       </c>
-      <c r="BN2" s="5">
+      <c r="BN2" s="5" t="n">
         <v>46285</v>
       </c>
-      <c r="BO2" s="5">
+      <c r="BO2" s="5" t="n">
         <v>46286</v>
       </c>
-      <c r="BP2" s="5">
+      <c r="BP2" s="5" t="n">
         <v>46287</v>
       </c>
-      <c r="BQ2" s="5">
+      <c r="BQ2" s="5" t="n">
         <v>46288</v>
       </c>
-      <c r="BR2" s="5">
+      <c r="BR2" s="5" t="n">
         <v>46289</v>
       </c>
-      <c r="BS2" s="5">
+      <c r="BS2" s="5" t="n">
         <v>46290</v>
       </c>
-      <c r="BT2" s="5">
+      <c r="BT2" s="5" t="n">
         <v>46291</v>
       </c>
-      <c r="BU2" s="5">
+      <c r="BU2" s="5" t="n">
         <v>46292</v>
       </c>
-      <c r="BV2" s="5">
+      <c r="BV2" s="5" t="n">
         <v>46293</v>
       </c>
-      <c r="BW2" s="5">
+      <c r="BW2" s="5" t="n">
         <v>46294</v>
       </c>
-      <c r="BX2" s="5">
+      <c r="BX2" s="5" t="n">
         <v>46295</v>
       </c>
-      <c r="BY2" s="5">
+      <c r="BY2" s="5" t="n">
         <v>46296</v>
       </c>
-      <c r="BZ2" s="5">
+      <c r="BZ2" s="5" t="n">
         <v>46297</v>
       </c>
-      <c r="CA2" s="5">
+      <c r="CA2" s="5" t="n">
         <v>46298</v>
       </c>
-      <c r="CB2" s="5">
+      <c r="CB2" s="5" t="n">
         <v>46299</v>
       </c>
-      <c r="CC2" s="5">
+      <c r="CC2" s="5" t="n">
         <v>46300</v>
       </c>
-      <c r="CD2" s="5">
+      <c r="CD2" s="5" t="n">
         <v>46301</v>
       </c>
-      <c r="CE2" s="5">
+      <c r="CE2" s="5" t="n">
         <v>46302</v>
       </c>
-      <c r="CF2" s="5">
+      <c r="CF2" s="5" t="n">
         <v>46303</v>
       </c>
-      <c r="CG2" s="5">
+      <c r="CG2" s="5" t="n">
         <v>46304</v>
       </c>
-      <c r="CH2" s="5">
+      <c r="CH2" s="5" t="n">
         <v>46305</v>
       </c>
-      <c r="CI2" s="5">
+      <c r="CI2" s="5" t="n">
         <v>46306</v>
       </c>
-      <c r="CJ2" s="5">
+      <c r="CJ2" s="5" t="n">
         <v>46307</v>
       </c>
-      <c r="CK2" s="5">
+      <c r="CK2" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="CL2" s="5">
+      <c r="CL2" s="5" t="n">
         <v>46309</v>
       </c>
-      <c r="CM2" s="5">
+      <c r="CM2" s="5" t="n">
         <v>46310</v>
       </c>
-      <c r="CN2" s="5">
+      <c r="CN2" s="5" t="n">
         <v>46311</v>
       </c>
-      <c r="CO2" s="5">
+      <c r="CO2" s="5" t="n">
         <v>46312</v>
       </c>
-      <c r="CP2" s="5">
+      <c r="CP2" s="5" t="n">
         <v>46313</v>
       </c>
-      <c r="CQ2" s="5">
+      <c r="CQ2" s="5" t="n">
         <v>46314</v>
       </c>
-      <c r="CR2" s="5">
+      <c r="CR2" s="5" t="n">
         <v>46315</v>
       </c>
-      <c r="CS2" s="5">
+      <c r="CS2" s="5" t="n">
         <v>46316</v>
       </c>
-      <c r="CT2" s="5">
+      <c r="CT2" s="5" t="n">
         <v>46317</v>
       </c>
-      <c r="CU2" s="5">
+      <c r="CU2" s="5" t="n">
         <v>46318</v>
       </c>
-      <c r="CV2" s="5">
+      <c r="CV2" s="5" t="n">
         <v>46319</v>
       </c>
-      <c r="CW2" s="5">
+      <c r="CW2" s="5" t="n">
         <v>46320</v>
       </c>
-      <c r="CX2" s="5">
+      <c r="CX2" s="5" t="n">
         <v>46321</v>
       </c>
-      <c r="CY2" s="5">
+      <c r="CY2" s="5" t="n">
         <v>46322</v>
       </c>
-      <c r="CZ2" s="5">
+      <c r="CZ2" s="5" t="n">
         <v>46323</v>
       </c>
-      <c r="DA2" s="5">
+      <c r="DA2" s="5" t="n">
         <v>46324</v>
       </c>
-      <c r="DB2" s="5">
+      <c r="DB2" s="5" t="n">
         <v>46325</v>
       </c>
-      <c r="DC2" s="5">
+      <c r="DC2" s="5" t="n">
         <v>46326</v>
       </c>
-      <c r="DD2" s="5">
+      <c r="DD2" s="5" t="n">
         <v>46327</v>
       </c>
-      <c r="DE2" s="5">
+      <c r="DE2" s="5" t="n">
         <v>46328</v>
       </c>
-      <c r="DF2" s="5">
+      <c r="DF2" s="5" t="n">
         <v>46329</v>
       </c>
-      <c r="DG2" s="5">
+      <c r="DG2" s="5" t="n">
         <v>46330</v>
       </c>
-      <c r="DH2" s="5">
+      <c r="DH2" s="5" t="n">
         <v>46331</v>
       </c>
-      <c r="DI2" s="5">
+      <c r="DI2" s="5" t="n">
         <v>46332</v>
       </c>
-      <c r="DJ2" s="5">
+      <c r="DJ2" s="5" t="n">
         <v>46333</v>
       </c>
-      <c r="DK2" s="5">
+      <c r="DK2" s="5" t="n">
         <v>46334</v>
       </c>
-      <c r="DL2" s="5">
+      <c r="DL2" s="5" t="n">
         <v>46335</v>
       </c>
-      <c r="DM2" s="5">
+      <c r="DM2" s="5" t="n">
         <v>46336</v>
       </c>
-      <c r="DN2" s="5">
+      <c r="DN2" s="5" t="n">
         <v>46337</v>
       </c>
-      <c r="DO2" s="5">
+      <c r="DO2" s="5" t="n">
         <v>46338</v>
       </c>
-      <c r="DP2" s="5">
+      <c r="DP2" s="5" t="n">
         <v>46339</v>
       </c>
-      <c r="DQ2" s="5">
+      <c r="DQ2" s="5" t="n">
         <v>46340</v>
       </c>
-      <c r="DR2" s="5">
+      <c r="DR2" s="5" t="n">
         <v>46341</v>
       </c>
-      <c r="DS2" s="5">
+      <c r="DS2" s="5" t="n">
         <v>46342</v>
       </c>
-      <c r="DT2" s="5">
+      <c r="DT2" s="5" t="n">
         <v>46343</v>
       </c>
-      <c r="DU2" s="5">
+      <c r="DU2" s="5" t="n">
         <v>46344</v>
       </c>
-      <c r="DV2" s="5">
+      <c r="DV2" s="5" t="n">
         <v>46345</v>
       </c>
-      <c r="DW2" s="5">
+      <c r="DW2" s="5" t="n">
         <v>46346</v>
       </c>
-      <c r="DX2" s="5">
+      <c r="DX2" s="5" t="n">
         <v>46347</v>
       </c>
-      <c r="DY2" s="5">
+      <c r="DY2" s="5" t="n">
         <v>46348</v>
       </c>
-      <c r="DZ2" s="5">
+      <c r="DZ2" s="5" t="n">
         <v>46349</v>
       </c>
-      <c r="EA2" s="5">
+      <c r="EA2" s="5" t="n">
         <v>46350</v>
       </c>
-      <c r="EB2" s="5">
+      <c r="EB2" s="5" t="n">
         <v>46351</v>
       </c>
-      <c r="EC2" s="5">
+      <c r="EC2" s="5" t="n">
         <v>46352</v>
       </c>
-      <c r="ED2" s="5">
+      <c r="ED2" s="5" t="n">
         <v>46353</v>
       </c>
-      <c r="EE2" s="5">
+      <c r="EE2" s="5" t="n">
         <v>46354</v>
       </c>
-      <c r="EF2" s="5">
+      <c r="EF2" s="5" t="n">
         <v>46355</v>
       </c>
-      <c r="EG2" s="5">
+      <c r="EG2" s="5" t="n">
         <v>46356</v>
       </c>
-      <c r="EH2" s="5">
+      <c r="EH2" s="5" t="n">
         <v>46357</v>
       </c>
-      <c r="EI2" s="5">
+      <c r="EI2" s="5" t="n">
         <v>46358</v>
       </c>
-      <c r="EJ2" s="5">
+      <c r="EJ2" s="5" t="n">
         <v>46359</v>
       </c>
-      <c r="EK2" s="5">
+      <c r="EK2" s="5" t="n">
         <v>46360</v>
       </c>
-      <c r="EL2" s="5">
+      <c r="EL2" s="5" t="n">
         <v>46361</v>
       </c>
-      <c r="EM2" s="5">
+      <c r="EM2" s="5" t="n">
         <v>46362</v>
       </c>
-      <c r="EN2" s="5">
+      <c r="EN2" s="5" t="n">
         <v>46363</v>
       </c>
-      <c r="EO2" s="5">
+      <c r="EO2" s="5" t="n">
         <v>46364</v>
       </c>
-      <c r="EP2" s="5">
+      <c r="EP2" s="5" t="n">
         <v>46365</v>
       </c>
-      <c r="EQ2" s="5">
+      <c r="EQ2" s="5" t="n">
         <v>46366</v>
       </c>
-      <c r="ER2" s="5">
+      <c r="ER2" s="5" t="n">
         <v>46367</v>
       </c>
-      <c r="ES2" s="5">
+      <c r="ES2" s="5" t="n">
         <v>46368</v>
       </c>
-      <c r="ET2" s="5">
+      <c r="ET2" s="5" t="n">
         <v>46369</v>
       </c>
-      <c r="EU2" s="5">
+      <c r="EU2" s="5" t="n">
         <v>46370</v>
       </c>
     </row>
-    <row r="3" spans="2:151" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="X3" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE3" s="9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="12"/>
-      <c r="K11" s="13"/>
-    </row>
-    <row r="12" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="12"/>
-    </row>
-    <row r="13" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="M13" s="10"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="12"/>
-    </row>
-    <row r="14" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="M14" s="10"/>
-      <c r="N14" s="12"/>
-    </row>
-    <row r="15" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="O15" s="10"/>
-      <c r="P15" s="11"/>
-      <c r="R15" s="10"/>
-      <c r="S15" s="12"/>
-    </row>
-    <row r="16" spans="2:151" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="T16" s="10"/>
-      <c r="U16" s="11"/>
-      <c r="V16" s="11"/>
-      <c r="W16" s="12"/>
-      <c r="Y16" s="13"/>
-    </row>
-    <row r="17" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="M17" s="10"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="R17" s="10"/>
-      <c r="S17" s="12"/>
-    </row>
-    <row r="18" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="T18" s="10"/>
-      <c r="U18" s="12"/>
-    </row>
-    <row r="19" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="U19" s="10"/>
-      <c r="V19" s="11"/>
-      <c r="W19" s="12"/>
-    </row>
-    <row r="20" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="Z20" s="10"/>
-      <c r="AA20" s="11"/>
-      <c r="AB20" s="11"/>
-      <c r="AC20" s="11"/>
-      <c r="AD20" s="12"/>
-    </row>
-    <row r="21" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="Z21" s="10"/>
-      <c r="AA21" s="12"/>
-    </row>
-    <row r="22" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z22" s="10"/>
-      <c r="AA22" s="11"/>
-      <c r="AB22" s="11"/>
-      <c r="AC22" s="11"/>
-      <c r="AD22" s="11"/>
-      <c r="AF22" s="13"/>
-    </row>
-    <row r="23" spans="2:32" outlineLevel="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="M23" s="10"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="12"/>
-    </row>
-    <row r="25" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="B25" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="6"/>
-    </row>
-    <row r="26" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="B26" s="7"/>
-    </row>
-    <row r="27" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="B27" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="6"/>
-    </row>
-    <row r="28" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="B28" s="7"/>
-    </row>
-    <row r="29" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="B29" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C29" s="6"/>
-    </row>
-    <row r="30" spans="2:32" x14ac:dyDescent="0.2">
-      <c r="B30" s="7"/>
+    <row r="3">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>MDFoods</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>◆ v1: User can see all products/contents</t>
+        </is>
+      </c>
+      <c r="X3" s="9" t="inlineStr">
+        <is>
+          <t>◆ v2: User can request a quote</t>
+        </is>
+      </c>
+      <c r="AE3" s="9" t="inlineStr">
+        <is>
+          <t>◆ v3: User can complete an order</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" outlineLevel="1" s="14">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>F-01: Master Layout</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+    </row>
+    <row r="5" outlineLevel="1" s="14">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>F-02: Landing Page (Home Page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" outlineLevel="1" s="14">
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>F-03: Product List by Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" outlineLevel="1" s="14">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>F-04: Product Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" outlineLevel="1" s="14">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>F-05: Product Search</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" outlineLevel="1" s="14">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>F-06: Static Pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" outlineLevel="1" s="14">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>F-07: Activities</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" outlineLevel="1" s="14">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>F-08: Registration</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="K11" s="13" t="n"/>
+    </row>
+    <row r="12" outlineLevel="1" s="14">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>F-09: Authentication</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="n"/>
+      <c r="I12" s="11" t="n"/>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="12" t="n"/>
+    </row>
+    <row r="13" outlineLevel="1" s="14">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>F-10: Profile Management</t>
+        </is>
+      </c>
+      <c r="M13" s="10" t="n"/>
+      <c r="N13" s="11" t="n"/>
+      <c r="O13" s="12" t="n"/>
+    </row>
+    <row r="14" outlineLevel="1" s="14">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>F-11: Addresses Management</t>
+        </is>
+      </c>
+      <c r="M14" s="10" t="n"/>
+      <c r="N14" s="12" t="n"/>
+    </row>
+    <row r="15" outlineLevel="1" s="14">
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>F-12: Company Information Management</t>
+        </is>
+      </c>
+      <c r="O15" s="10" t="n"/>
+      <c r="P15" s="11" t="n"/>
+      <c r="R15" s="10" t="n"/>
+      <c r="S15" s="12" t="n"/>
+    </row>
+    <row r="16" outlineLevel="1" s="14">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>F-13: Company Member/Permission Management</t>
+        </is>
+      </c>
+      <c r="T16" s="10" t="n"/>
+      <c r="U16" s="11" t="n"/>
+      <c r="V16" s="11" t="n"/>
+      <c r="W16" s="12" t="n"/>
+      <c r="Y16" s="13" t="n"/>
+    </row>
+    <row r="17" outlineLevel="1" s="14">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>F-14: Shopping Cart</t>
+        </is>
+      </c>
+      <c r="M17" s="10" t="n"/>
+      <c r="N17" s="11" t="n"/>
+      <c r="O17" s="11" t="n"/>
+      <c r="P17" s="11" t="n"/>
+      <c r="R17" s="10" t="n"/>
+      <c r="S17" s="12" t="n"/>
+    </row>
+    <row r="18" outlineLevel="1" s="14">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>F-15: Request Quote Process</t>
+        </is>
+      </c>
+      <c r="T18" s="10" t="n"/>
+      <c r="U18" s="12" t="n"/>
+    </row>
+    <row r="19" outlineLevel="1" s="14">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>F-16: Quote Management</t>
+        </is>
+      </c>
+      <c r="U19" s="10" t="n"/>
+      <c r="V19" s="11" t="n"/>
+      <c r="W19" s="12" t="n"/>
+    </row>
+    <row r="20" outlineLevel="1" s="14">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>F-17: Order &amp; Payment</t>
+        </is>
+      </c>
+      <c r="Z20" s="10" t="n"/>
+      <c r="AA20" s="11" t="n"/>
+      <c r="AB20" s="11" t="n"/>
+      <c r="AC20" s="11" t="n"/>
+      <c r="AD20" s="12" t="n"/>
+    </row>
+    <row r="21" outlineLevel="1" s="14">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>F-18: Orders Management</t>
+        </is>
+      </c>
+      <c r="Z21" s="10" t="n"/>
+      <c r="AA21" s="12" t="n"/>
+    </row>
+    <row r="22" outlineLevel="1" s="14">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>F-19: In-App Messages and Notification</t>
+        </is>
+      </c>
+      <c r="Z22" s="10" t="n"/>
+      <c r="AA22" s="11" t="n"/>
+      <c r="AB22" s="11" t="n"/>
+      <c r="AC22" s="11" t="n"/>
+      <c r="AD22" s="11" t="n"/>
+      <c r="AF22" s="13" t="n"/>
+    </row>
+    <row r="23" outlineLevel="1" s="14">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>F-20: Password Recovery</t>
+        </is>
+      </c>
+      <c r="M23" s="10" t="n"/>
+      <c r="N23" s="11" t="n"/>
+      <c r="O23" s="12" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Odeli</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>LFarm</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:EU10 C11:C12 J11:EU12 S13:EU14 C13:J23 Q13:Q26 V15:EU15 X16:EU17 R17:W17 V18:EU18 X19:EU19 AF20:EU21 S20:X22 AE20:AE22 AL22:EU22 S23:EU23 C24:P26 R24:EU26 C27:EU1048576">
-    <cfRule type="expression" dxfId="7" priority="3">
+  <conditionalFormatting sqref="C2:EU10 C11:C12 C13:J23 C24:P26 C27:EU1048576 J11:EU12 Q13:Q26 R17:W17 R24:EU26 S13:EU14 S20:X22 S23:EU23 V15:EU15 V18:EU18 X16:EU17 X19:EU19 AE20:AE22 AF20:EU21 AL22:EU22">
+    <cfRule type="expression" priority="3" dxfId="0">
       <formula>WEEKDAY(C$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:I11 T16:W16 T18:U18 Z20:AD21">
-    <cfRule type="expression" dxfId="6" priority="11">
+    <cfRule type="expression" priority="11" dxfId="0">
       <formula>WEEKDAY(D$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F12:I12 M13:P14 R13:R14 M15:N15 R16 M16:P23 R18:R23">
-    <cfRule type="expression" dxfId="5" priority="13">
+  <conditionalFormatting sqref="F12:I12 M13:P14 M15:N15 M16:P23 R13:R14 R16 R18:R23">
+    <cfRule type="expression" priority="13" dxfId="0">
       <formula>WEEKDAY(D$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15:P15">
-    <cfRule type="expression" dxfId="4" priority="5">
+    <cfRule type="expression" priority="5" dxfId="0">
       <formula>WEEKDAY(R$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R15:S15">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>WEEKDAY(R$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U19:W19">
-    <cfRule type="expression" dxfId="2" priority="7">
+    <cfRule type="expression" priority="7" dxfId="0">
       <formula>WEEKDAY(R$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z22:AD22">
-    <cfRule type="expression" dxfId="1" priority="9">
+    <cfRule type="expression" priority="9" dxfId="0">
       <formula>WEEKDAY(AF$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF22">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>WEEKDAY(AF$2)=1</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="B7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="B8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B9" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B10" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B11" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="B13" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="B14" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="B15" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B16" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B17" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B18" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B19" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B20" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B21" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B22" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B23" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:EU7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="2.6640625" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="151" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col width="2.6640625" customWidth="1" style="14" min="1" max="1"/>
+    <col width="18.83203125" customWidth="1" style="14" min="2" max="2"/>
+    <col width="5.83203125" bestFit="1" customWidth="1" style="14" min="3" max="151"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:151" ht="13" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:151" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="5">
+    <row r="1" ht="13" customHeight="1" s="14"/>
+    <row r="2" customFormat="1" s="3">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>46222</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="5" t="n">
         <v>46223</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="5" t="n">
         <v>46224</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="5" t="n">
         <v>46225</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="5" t="n">
         <v>46226</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="5" t="n">
         <v>46227</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="5" t="n">
         <v>46228</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="5" t="n">
         <v>46229</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="5" t="n">
         <v>46230</v>
       </c>
-      <c r="L2" s="5">
+      <c r="L2" s="5" t="n">
         <v>46231</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2" s="5" t="n">
         <v>46232</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="5" t="n">
         <v>46233</v>
       </c>
-      <c r="O2" s="5">
+      <c r="O2" s="5" t="n">
         <v>46234</v>
       </c>
-      <c r="P2" s="5">
+      <c r="P2" s="5" t="n">
         <v>46235</v>
       </c>
-      <c r="Q2" s="5">
+      <c r="Q2" s="5" t="n">
         <v>46236</v>
       </c>
-      <c r="R2" s="5">
+      <c r="R2" s="5" t="n">
         <v>46237</v>
       </c>
-      <c r="S2" s="5">
+      <c r="S2" s="5" t="n">
         <v>46238</v>
       </c>
-      <c r="T2" s="5">
+      <c r="T2" s="5" t="n">
         <v>46239</v>
       </c>
-      <c r="U2" s="5">
+      <c r="U2" s="5" t="n">
         <v>46240</v>
       </c>
-      <c r="V2" s="5">
+      <c r="V2" s="5" t="n">
         <v>46241</v>
       </c>
-      <c r="W2" s="5">
+      <c r="W2" s="5" t="n">
         <v>46242</v>
       </c>
-      <c r="X2" s="5">
+      <c r="X2" s="5" t="n">
         <v>46243</v>
       </c>
-      <c r="Y2" s="5">
+      <c r="Y2" s="5" t="n">
         <v>46244</v>
       </c>
-      <c r="Z2" s="5">
+      <c r="Z2" s="5" t="n">
         <v>46245</v>
       </c>
-      <c r="AA2" s="5">
+      <c r="AA2" s="5" t="n">
         <v>46246</v>
       </c>
-      <c r="AB2" s="5">
+      <c r="AB2" s="5" t="n">
         <v>46247</v>
       </c>
-      <c r="AC2" s="5">
+      <c r="AC2" s="5" t="n">
         <v>46248</v>
       </c>
-      <c r="AD2" s="5">
+      <c r="AD2" s="5" t="n">
         <v>46249</v>
       </c>
-      <c r="AE2" s="5">
+      <c r="AE2" s="5" t="n">
         <v>46250</v>
       </c>
-      <c r="AF2" s="5">
+      <c r="AF2" s="5" t="n">
         <v>46251</v>
       </c>
-      <c r="AG2" s="5">
+      <c r="AG2" s="5" t="n">
         <v>46252</v>
       </c>
-      <c r="AH2" s="5">
+      <c r="AH2" s="5" t="n">
         <v>46253</v>
       </c>
-      <c r="AI2" s="5">
+      <c r="AI2" s="5" t="n">
         <v>46254</v>
       </c>
-      <c r="AJ2" s="5">
+      <c r="AJ2" s="5" t="n">
         <v>46255</v>
       </c>
-      <c r="AK2" s="5">
+      <c r="AK2" s="5" t="n">
         <v>46256</v>
       </c>
-      <c r="AL2" s="5">
+      <c r="AL2" s="5" t="n">
         <v>46257</v>
       </c>
-      <c r="AM2" s="5">
+      <c r="AM2" s="5" t="n">
         <v>46258</v>
       </c>
-      <c r="AN2" s="5">
+      <c r="AN2" s="5" t="n">
         <v>46259</v>
       </c>
-      <c r="AO2" s="5">
+      <c r="AO2" s="5" t="n">
         <v>46260</v>
       </c>
-      <c r="AP2" s="5">
+      <c r="AP2" s="5" t="n">
         <v>46261</v>
       </c>
-      <c r="AQ2" s="5">
+      <c r="AQ2" s="5" t="n">
         <v>46262</v>
       </c>
-      <c r="AR2" s="5">
+      <c r="AR2" s="5" t="n">
         <v>46263</v>
       </c>
-      <c r="AS2" s="5">
+      <c r="AS2" s="5" t="n">
         <v>46264</v>
       </c>
-      <c r="AT2" s="5">
+      <c r="AT2" s="5" t="n">
         <v>46265</v>
       </c>
-      <c r="AU2" s="5">
+      <c r="AU2" s="5" t="n">
         <v>46266</v>
       </c>
-      <c r="AV2" s="5">
+      <c r="AV2" s="5" t="n">
         <v>46267</v>
       </c>
-      <c r="AW2" s="5">
+      <c r="AW2" s="5" t="n">
         <v>46268</v>
       </c>
-      <c r="AX2" s="5">
+      <c r="AX2" s="5" t="n">
         <v>46269</v>
       </c>
-      <c r="AY2" s="5">
+      <c r="AY2" s="5" t="n">
         <v>46270</v>
       </c>
-      <c r="AZ2" s="5">
+      <c r="AZ2" s="5" t="n">
         <v>46271</v>
       </c>
-      <c r="BA2" s="5">
+      <c r="BA2" s="5" t="n">
         <v>46272</v>
       </c>
-      <c r="BB2" s="5">
+      <c r="BB2" s="5" t="n">
         <v>46273</v>
       </c>
-      <c r="BC2" s="5">
+      <c r="BC2" s="5" t="n">
         <v>46274</v>
       </c>
-      <c r="BD2" s="5">
+      <c r="BD2" s="5" t="n">
         <v>46275</v>
       </c>
-      <c r="BE2" s="5">
+      <c r="BE2" s="5" t="n">
         <v>46276</v>
       </c>
-      <c r="BF2" s="5">
+      <c r="BF2" s="5" t="n">
         <v>46277</v>
       </c>
-      <c r="BG2" s="5">
+      <c r="BG2" s="5" t="n">
         <v>46278</v>
       </c>
-      <c r="BH2" s="5">
+      <c r="BH2" s="5" t="n">
         <v>46279</v>
       </c>
-      <c r="BI2" s="5">
+      <c r="BI2" s="5" t="n">
         <v>46280</v>
       </c>
-      <c r="BJ2" s="5">
+      <c r="BJ2" s="5" t="n">
         <v>46281</v>
       </c>
-      <c r="BK2" s="5">
+      <c r="BK2" s="5" t="n">
         <v>46282</v>
       </c>
-      <c r="BL2" s="5">
+      <c r="BL2" s="5" t="n">
         <v>46283</v>
       </c>
-      <c r="BM2" s="5">
+      <c r="BM2" s="5" t="n">
         <v>46284</v>
       </c>
-      <c r="BN2" s="5">
+      <c r="BN2" s="5" t="n">
         <v>46285</v>
       </c>
-      <c r="BO2" s="5">
+      <c r="BO2" s="5" t="n">
         <v>46286</v>
       </c>
-      <c r="BP2" s="5">
+      <c r="BP2" s="5" t="n">
         <v>46287</v>
       </c>
-      <c r="BQ2" s="5">
+      <c r="BQ2" s="5" t="n">
         <v>46288</v>
       </c>
-      <c r="BR2" s="5">
+      <c r="BR2" s="5" t="n">
         <v>46289</v>
       </c>
-      <c r="BS2" s="5">
+      <c r="BS2" s="5" t="n">
         <v>46290</v>
       </c>
-      <c r="BT2" s="5">
+      <c r="BT2" s="5" t="n">
         <v>46291</v>
       </c>
-      <c r="BU2" s="5">
+      <c r="BU2" s="5" t="n">
         <v>46292</v>
       </c>
-      <c r="BV2" s="5">
+      <c r="BV2" s="5" t="n">
         <v>46293</v>
       </c>
-      <c r="BW2" s="5">
+      <c r="BW2" s="5" t="n">
         <v>46294</v>
       </c>
-      <c r="BX2" s="5">
+      <c r="BX2" s="5" t="n">
         <v>46295</v>
       </c>
-      <c r="BY2" s="5">
+      <c r="BY2" s="5" t="n">
         <v>46296</v>
       </c>
-      <c r="BZ2" s="5">
+      <c r="BZ2" s="5" t="n">
         <v>46297</v>
       </c>
-      <c r="CA2" s="5">
+      <c r="CA2" s="5" t="n">
         <v>46298</v>
       </c>
-      <c r="CB2" s="5">
+      <c r="CB2" s="5" t="n">
         <v>46299</v>
       </c>
-      <c r="CC2" s="5">
+      <c r="CC2" s="5" t="n">
         <v>46300</v>
       </c>
-      <c r="CD2" s="5">
+      <c r="CD2" s="5" t="n">
         <v>46301</v>
       </c>
-      <c r="CE2" s="5">
+      <c r="CE2" s="5" t="n">
         <v>46302</v>
       </c>
-      <c r="CF2" s="5">
+      <c r="CF2" s="5" t="n">
         <v>46303</v>
       </c>
-      <c r="CG2" s="5">
+      <c r="CG2" s="5" t="n">
         <v>46304</v>
       </c>
-      <c r="CH2" s="5">
+      <c r="CH2" s="5" t="n">
         <v>46305</v>
       </c>
-      <c r="CI2" s="5">
+      <c r="CI2" s="5" t="n">
         <v>46306</v>
       </c>
-      <c r="CJ2" s="5">
+      <c r="CJ2" s="5" t="n">
         <v>46307</v>
       </c>
-      <c r="CK2" s="5">
+      <c r="CK2" s="5" t="n">
         <v>46308</v>
       </c>
-      <c r="CL2" s="5">
+      <c r="CL2" s="5" t="n">
         <v>46309</v>
       </c>
-      <c r="CM2" s="5">
+      <c r="CM2" s="5" t="n">
         <v>46310</v>
       </c>
-      <c r="CN2" s="5">
+      <c r="CN2" s="5" t="n">
         <v>46311</v>
       </c>
-      <c r="CO2" s="5">
+      <c r="CO2" s="5" t="n">
         <v>46312</v>
       </c>
-      <c r="CP2" s="5">
+      <c r="CP2" s="5" t="n">
         <v>46313</v>
       </c>
-      <c r="CQ2" s="5">
+      <c r="CQ2" s="5" t="n">
         <v>46314</v>
       </c>
-      <c r="CR2" s="5">
+      <c r="CR2" s="5" t="n">
         <v>46315</v>
       </c>
-      <c r="CS2" s="5">
+      <c r="CS2" s="5" t="n">
         <v>46316</v>
       </c>
-      <c r="CT2" s="5">
+      <c r="CT2" s="5" t="n">
         <v>46317</v>
       </c>
-      <c r="CU2" s="5">
+      <c r="CU2" s="5" t="n">
         <v>46318</v>
       </c>
-      <c r="CV2" s="5">
+      <c r="CV2" s="5" t="n">
         <v>46319</v>
       </c>
-      <c r="CW2" s="5">
+      <c r="CW2" s="5" t="n">
         <v>46320</v>
       </c>
-      <c r="CX2" s="5">
+      <c r="CX2" s="5" t="n">
         <v>46321</v>
       </c>
-      <c r="CY2" s="5">
+      <c r="CY2" s="5" t="n">
         <v>46322</v>
       </c>
-      <c r="CZ2" s="5">
+      <c r="CZ2" s="5" t="n">
         <v>46323</v>
       </c>
-      <c r="DA2" s="5">
+      <c r="DA2" s="5" t="n">
         <v>46324</v>
       </c>
-      <c r="DB2" s="5">
+      <c r="DB2" s="5" t="n">
         <v>46325</v>
       </c>
-      <c r="DC2" s="5">
+      <c r="DC2" s="5" t="n">
         <v>46326</v>
       </c>
-      <c r="DD2" s="5">
+      <c r="DD2" s="5" t="n">
         <v>46327</v>
       </c>
-      <c r="DE2" s="5">
+      <c r="DE2" s="5" t="n">
         <v>46328</v>
       </c>
-      <c r="DF2" s="5">
+      <c r="DF2" s="5" t="n">
         <v>46329</v>
       </c>
-      <c r="DG2" s="5">
+      <c r="DG2" s="5" t="n">
         <v>46330</v>
       </c>
-      <c r="DH2" s="5">
+      <c r="DH2" s="5" t="n">
         <v>46331</v>
       </c>
-      <c r="DI2" s="5">
+      <c r="DI2" s="5" t="n">
         <v>46332</v>
       </c>
-      <c r="DJ2" s="5">
+      <c r="DJ2" s="5" t="n">
         <v>46333</v>
       </c>
-      <c r="DK2" s="5">
+      <c r="DK2" s="5" t="n">
         <v>46334</v>
       </c>
-      <c r="DL2" s="5">
+      <c r="DL2" s="5" t="n">
         <v>46335</v>
       </c>
-      <c r="DM2" s="5">
+      <c r="DM2" s="5" t="n">
         <v>46336</v>
       </c>
-      <c r="DN2" s="5">
+      <c r="DN2" s="5" t="n">
         <v>46337</v>
       </c>
-      <c r="DO2" s="5">
+      <c r="DO2" s="5" t="n">
         <v>46338</v>
       </c>
-      <c r="DP2" s="5">
+      <c r="DP2" s="5" t="n">
         <v>46339</v>
       </c>
-      <c r="DQ2" s="5">
+      <c r="DQ2" s="5" t="n">
         <v>46340</v>
       </c>
-      <c r="DR2" s="5">
+      <c r="DR2" s="5" t="n">
         <v>46341</v>
       </c>
-      <c r="DS2" s="5">
+      <c r="DS2" s="5" t="n">
         <v>46342</v>
       </c>
-      <c r="DT2" s="5">
+      <c r="DT2" s="5" t="n">
         <v>46343</v>
       </c>
-      <c r="DU2" s="5">
+      <c r="DU2" s="5" t="n">
         <v>46344</v>
       </c>
-      <c r="DV2" s="5">
+      <c r="DV2" s="5" t="n">
         <v>46345</v>
       </c>
-      <c r="DW2" s="5">
+      <c r="DW2" s="5" t="n">
         <v>46346</v>
       </c>
-      <c r="DX2" s="5">
+      <c r="DX2" s="5" t="n">
         <v>46347</v>
       </c>
-      <c r="DY2" s="5">
+      <c r="DY2" s="5" t="n">
         <v>46348</v>
       </c>
-      <c r="DZ2" s="5">
+      <c r="DZ2" s="5" t="n">
         <v>46349</v>
       </c>
-      <c r="EA2" s="5">
+      <c r="EA2" s="5" t="n">
         <v>46350</v>
       </c>
-      <c r="EB2" s="5">
+      <c r="EB2" s="5" t="n">
         <v>46351</v>
       </c>
-      <c r="EC2" s="5">
+      <c r="EC2" s="5" t="n">
         <v>46352</v>
       </c>
-      <c r="ED2" s="5">
+      <c r="ED2" s="5" t="n">
         <v>46353</v>
       </c>
-      <c r="EE2" s="5">
+      <c r="EE2" s="5" t="n">
         <v>46354</v>
       </c>
-      <c r="EF2" s="5">
+      <c r="EF2" s="5" t="n">
         <v>46355</v>
       </c>
-      <c r="EG2" s="5">
+      <c r="EG2" s="5" t="n">
         <v>46356</v>
       </c>
-      <c r="EH2" s="5">
+      <c r="EH2" s="5" t="n">
         <v>46357</v>
       </c>
-      <c r="EI2" s="5">
+      <c r="EI2" s="5" t="n">
         <v>46358</v>
       </c>
-      <c r="EJ2" s="5">
+      <c r="EJ2" s="5" t="n">
         <v>46359</v>
       </c>
-      <c r="EK2" s="5">
+      <c r="EK2" s="5" t="n">
         <v>46360</v>
       </c>
-      <c r="EL2" s="5">
+      <c r="EL2" s="5" t="n">
         <v>46361</v>
       </c>
-      <c r="EM2" s="5">
+      <c r="EM2" s="5" t="n">
         <v>46362</v>
       </c>
-      <c r="EN2" s="5">
+      <c r="EN2" s="5" t="n">
         <v>46363</v>
       </c>
-      <c r="EO2" s="5">
+      <c r="EO2" s="5" t="n">
         <v>46364</v>
       </c>
-      <c r="EP2" s="5">
+      <c r="EP2" s="5" t="n">
         <v>46365</v>
       </c>
-      <c r="EQ2" s="5">
+      <c r="EQ2" s="5" t="n">
         <v>46366</v>
       </c>
-      <c r="ER2" s="5">
+      <c r="ER2" s="5" t="n">
         <v>46367</v>
       </c>
-      <c r="ES2" s="5">
+      <c r="ES2" s="5" t="n">
         <v>46368</v>
       </c>
-      <c r="ET2" s="5">
+      <c r="ET2" s="5" t="n">
         <v>46369</v>
       </c>
-      <c r="EU2" s="5">
+      <c r="EU2" s="5" t="n">
         <v>46370</v>
       </c>
     </row>
-    <row r="3" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3"/>
-      <c r="B3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="15">
+    <row r="3" s="14">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>An Nguyen 1</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4"/>
-      <c r="B4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="14">
+    <row r="4" s="14">
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Khuong Nguyen 1</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5"/>
-      <c r="B5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="14">
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" s="14">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Phat Phan 1</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6"/>
-      <c r="B6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E6" s="14">
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" s="14">
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Phat Phan 2</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:151" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7"/>
-      <c r="B7" s="1" t="s">
-        <v>33</v>
+      <c r="F6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" s="14">
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Phat Ngo 1</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>